<commit_message>
Menú infantil (Chiken Junior), invitados renombrados a 4 cupos y Sra. Sandra Carvajal
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="49.140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -892,21 +892,21 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Sr. Andrey Vergara y esposa</t>
+          <t>Sr. Andrey Vergara, esposa, hijo e hija</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Sr. Fernando Valderrama y esposa</t>
+          <t>Sr. Fernando Valderrama, esposa, hijo e hija</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -1137,6 +1137,16 @@
       </c>
       <c r="B51" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sra. Sandra Carvajal</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lista de invitados: Martha Saavedra a 1 cupo y 5 invitados nuevos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="49.140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1146,6 +1146,56 @@
         </is>
       </c>
       <c r="B52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sr. Gabriel Pérez y esposa</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Sr. Nelson Botero y esposa</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Sr. Ricardo Forero y esposa</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Sr. Romel Guzmán y esposa</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Srta. Wendy Trujillo</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sr. Nelson Botero, esposa e hija: 3 cupos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -1162,11 +1162,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Sr. Nelson Botero y esposa</t>
+          <t>Sr. Nelson Botero, esposa e hija</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">

</xml_diff>

<commit_message>
Sr. Fernando Valderrama y esposa: 2 cupos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -902,11 +902,11 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Sr. Fernando Valderrama, esposa, hijo e hija</t>
+          <t>Sr. Fernando Valderrama y esposa</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Sr. Gabriel Pérez, esposa e hijo: 3 cupos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -1152,11 +1152,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sr. Gabriel Pérez y esposa</t>
+          <t>Sr. Gabriel Pérez, esposa e hijo</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">

</xml_diff>

<commit_message>
Sr. Fernando Valderrama, esposa e hijos: 4 cupos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -902,11 +902,11 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Sr. Fernando Valderrama y esposa</t>
+          <t>Sr. Fernando Valderrama, esposa e hijos</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Romel Guzmán, esposa e hija (3 cupos) y 3 invitadas Montoya
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="49.140625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -1182,11 +1182,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Sr. Romel Guzmán y esposa</t>
+          <t>Sr. Romel Guzmán, esposa e hija</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
@@ -1196,6 +1196,36 @@
         </is>
       </c>
       <c r="B57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Yolanda Montoya</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Luz Montoya</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Marina Montoya</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sr. Gabriel Pérez, esposa e hijos: 4 cupos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6W6J7bQRWPHU2XBCQF8z
</commit_message>
<xml_diff>
--- a/INVITADOS.xlsx
+++ b/INVITADOS.xlsx
@@ -1152,11 +1152,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sr. Gabriel Pérez, esposa e hijo</t>
+          <t>Sr. Gabriel Pérez, esposa e hijos</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54">

</xml_diff>